<commit_message>
feat: verify rule CG0208 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000002/negative/01/data/unit-test-coreid-CG0208-negative01.xlsx
+++ b/rules/CORE-000002/negative/01/data/unit-test-coreid-CG0208-negative01.xlsx
@@ -607,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,6 +639,52 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>se.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SESTDTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>se.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SESTDTC</t>
         </is>
       </c>
     </row>

</xml_diff>